<commit_message>
switched cronjob to windows task scheduler and one liner for running daily
</commit_message>
<xml_diff>
--- a/config/products.xlsx
+++ b/config/products.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,6 +485,364 @@
           <t>cierre_crop_name</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>aguacate</t>
+        </is>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>aguacate</t>
+        </is>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>133</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Aguacate</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>tomate</t>
+        </is>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>jitomate|tomate</t>
+        </is>
+      </c>
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>elote</t>
+        </is>
+      </c>
+      <c r="C4" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>elote por pieza|elote</t>
+        </is>
+      </c>
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>zanahoria</t>
+        </is>
+      </c>
+      <c r="C5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>zanahoria</t>
+        </is>
+      </c>
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>cebolla</t>
+        </is>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>cebolla</t>
+        </is>
+      </c>
+      <c r="E6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>chile_jalapeno</t>
+        </is>
+      </c>
+      <c r="C7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>chile jalapeno por kilo|chile jalapeno|jalapeno</t>
+        </is>
+      </c>
+      <c r="E7" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>limon</t>
+        </is>
+      </c>
+      <c r="C8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>limon</t>
+        </is>
+      </c>
+      <c r="E8" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+      <c r="K8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>platano</t>
+        </is>
+      </c>
+      <c r="C9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>platano</t>
+        </is>
+      </c>
+      <c r="E9" t="b">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>mango</t>
+        </is>
+      </c>
+      <c r="C10" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>mango</t>
+        </is>
+      </c>
+      <c r="E10" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>papa</t>
+        </is>
+      </c>
+      <c r="C11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>papa</t>
+        </is>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>233</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: remove outdated aguacate data files and add batch summary JSON
- Deleted the old Excel files for aguacate data (2024) as they are no longer needed.
- Introduced a new JSON file (`batch_summary.json`) to summarize batch processing results for multiple crops.
- Enhanced the `build_master_price_workbook.py` script to support additional column mappings and fallback mechanisms for reading Excel sheets.
- Added a new script (`fetch_cierre_batch.py`) to fetch and process Cierre Agricola data for multiple products and years, including error handling and logging.
- Updated the `cierre_agricola_requests.py` to ensure proper metadata handling in reports.
- Added unit tests to validate the new functionality and ensure compatibility with existing workflows.
</commit_message>
<xml_diff>
--- a/config/products.xlsx
+++ b/config/products.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22992" windowHeight="9168"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22990" windowHeight="9170"/>
   </bookViews>
   <sheets>
     <sheet name="productos" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="49">
   <si>
     <t>activo</t>
   </si>
@@ -67,15 +67,9 @@
     <t>Aguacate</t>
   </si>
   <si>
-    <t>tomate</t>
-  </si>
-  <si>
     <t>jitomate|tomate</t>
   </si>
   <si>
-    <t>elote</t>
-  </si>
-  <si>
     <t>elote por pieza|elote</t>
   </si>
   <si>
@@ -85,9 +79,6 @@
     <t>cebolla</t>
   </si>
   <si>
-    <t>chile_jalapeno</t>
-  </si>
-  <si>
     <t>chile jalapeno por kilo|chile jalapeno|jalapeno</t>
   </si>
   <si>
@@ -149,6 +140,33 @@
   </si>
   <si>
     <t>mango ataulfo</t>
+  </si>
+  <si>
+    <t>Limón</t>
+  </si>
+  <si>
+    <t>Plátano</t>
+  </si>
+  <si>
+    <t>Mango</t>
+  </si>
+  <si>
+    <t>Papa</t>
+  </si>
+  <si>
+    <t>Cebolla</t>
+  </si>
+  <si>
+    <t>Zanahoria</t>
+  </si>
+  <si>
+    <t>Elote</t>
+  </si>
+  <si>
+    <t>Tomate rojo</t>
+  </si>
+  <si>
+    <t>Chile verde</t>
   </si>
 </sst>
 </file>
@@ -512,12 +530,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -558,12 +576,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="b">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -599,24 +617,24 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="b">
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" t="b">
-        <v>1</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
       <c r="E3" t="b">
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G3" t="b">
         <v>1</v>
@@ -637,24 +655,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="b">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
@@ -675,24 +693,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="b">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
@@ -713,24 +731,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="b">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
@@ -751,24 +769,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="b">
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
@@ -789,24 +807,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="b">
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="C8" t="b">
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G8" t="b">
         <v>1</v>
@@ -827,24 +845,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="b">
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
@@ -865,24 +883,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="b">
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="C10" t="b">
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
@@ -903,24 +921,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="b">
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="C11" t="b">
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E11" t="b">
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G11" t="b">
         <v>1</v>
@@ -949,118 +967,118 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Enhance Walmart produce scraper with configurable search terms
- Added functionality to load search terms from an Excel workbook, allowing for dynamic configuration of product search terms.
- Introduced a new function `load_search_terms_from_workbook` to parse the configuration file and validate required columns.
- Updated `item_to_record` to reject conflicting inferred products based on configured crops.
- Modified the main execution flow to utilize the loaded search terms if a configuration file is provided.
- Added unit tests to ensure the new functionality works as expected, including tests for loading search terms and handling conflicts.
</commit_message>
<xml_diff>
--- a/config/products.xlsx
+++ b/config/products.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="48">
   <si>
     <t>activo</t>
   </si>
@@ -89,9 +89,6 @@
   </si>
   <si>
     <t>mango</t>
-  </si>
-  <si>
-    <t>papa</t>
   </si>
   <si>
     <t>campo</t>
@@ -622,7 +619,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -654,13 +651,16 @@
       <c r="L3" t="b">
         <v>0</v>
       </c>
+      <c r="M3" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="b">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
@@ -692,13 +692,16 @@
       <c r="L4" t="b">
         <v>0</v>
       </c>
+      <c r="M4" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="b">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
@@ -730,13 +733,16 @@
       <c r="L5" t="b">
         <v>0</v>
       </c>
+      <c r="M5" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="b">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
@@ -768,13 +774,16 @@
       <c r="L6" t="b">
         <v>0</v>
       </c>
+      <c r="M6" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="b">
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
@@ -806,13 +815,16 @@
       <c r="L7" t="b">
         <v>0</v>
       </c>
+      <c r="M7" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="b">
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C8" t="b">
         <v>1</v>
@@ -844,13 +856,16 @@
       <c r="L8" t="b">
         <v>0</v>
       </c>
+      <c r="M8" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="b">
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
@@ -882,13 +897,16 @@
       <c r="L9" t="b">
         <v>0</v>
       </c>
+      <c r="M9" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="b">
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C10" t="b">
         <v>1</v>
@@ -900,7 +918,7 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
@@ -920,25 +938,28 @@
       <c r="L10" t="b">
         <v>0</v>
       </c>
+      <c r="M10" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="b">
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C11" t="b">
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="E11" t="b">
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G11" t="b">
         <v>1</v>
@@ -957,6 +978,9 @@
       </c>
       <c r="L11" t="b">
         <v>0</v>
+      </c>
+      <c r="M11" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -971,10 +995,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -982,7 +1006,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -990,7 +1014,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -998,7 +1022,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -1006,7 +1030,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -1014,7 +1038,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -1022,7 +1046,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -1030,7 +1054,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -1038,7 +1062,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -1046,7 +1070,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -1054,7 +1078,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -1062,7 +1086,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -1070,7 +1094,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -1078,7 +1102,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>